<commit_message>
new code for VIP 2025
</commit_message>
<xml_diff>
--- a/data/vip2025.xlsx
+++ b/data/vip2025.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E068C319-0CE6-DD4F-81E0-7F8FF9A07FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDA950C-A54E-A746-8BCB-FD998D3DC574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1300" windowWidth="20920" windowHeight="19440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nights" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="23">
   <si>
     <t>lights</t>
   </si>
@@ -53,6 +53,42 @@
   </si>
   <si>
     <t>Viki</t>
+  </si>
+  <si>
+    <t>Leandro</t>
+  </si>
+  <si>
+    <t>Calvin O.</t>
+  </si>
+  <si>
+    <t>Jonny</t>
+  </si>
+  <si>
+    <t>Sidar</t>
+  </si>
+  <si>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>Rob</t>
+  </si>
+  <si>
+    <t>Nico</t>
+  </si>
+  <si>
+    <t>Lennert</t>
+  </si>
+  <si>
+    <t>Xander</t>
+  </si>
+  <si>
+    <t>Calvin S.</t>
+  </si>
+  <si>
+    <t>Olli</t>
+  </si>
+  <si>
+    <t>Jimi</t>
   </si>
 </sst>
 </file>
@@ -74,12 +110,24 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -124,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -141,13 +189,8 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,7 +496,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" style="1" bestFit="1" customWidth="1"/>
@@ -461,7 +504,7 @@
     <col min="12" max="12" width="12.5" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
@@ -496,131 +539,180 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="6"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="8"/>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="5">
+        <v>2</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="8"/>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" s="5">
+        <v>2</v>
+      </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="8"/>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="5">
+        <v>2</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="6"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="8"/>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L5" s="5">
+        <v>3</v>
+      </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="8"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="6"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="8"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="6"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="8"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="6"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="8"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="6"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="8"/>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L6" s="5">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
remove Pair clase, time testing, compare to aytorakel
</commit_message>
<xml_diff>
--- a/data/vip2025.xlsx
+++ b/data/vip2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{03B1CF5B-EF22-AF4A-B113-C0E57384EF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805FC4C3-AFAA-9041-8519-5BC3B6164E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="760" windowWidth="29620" windowHeight="13820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="760" windowWidth="33720" windowHeight="17820" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>
@@ -19,12 +19,11 @@
     <sheet name="Solution" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="28">
   <si>
     <t>left</t>
   </si>
@@ -108,12 +107,6 @@
   </si>
   <si>
     <t>result</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>true</t>
   </si>
 </sst>
 </file>
@@ -1478,7 +1471,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -1508,8 +1501,8 @@
       <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
-        <v>28</v>
+      <c r="D2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1522,8 +1515,8 @@
       <c r="C3" t="s">
         <v>24</v>
       </c>
-      <c r="D3" t="s">
-        <v>29</v>
+      <c r="D3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1536,8 +1529,8 @@
       <c r="C4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" t="s">
-        <v>28</v>
+      <c r="D4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1550,8 +1543,8 @@
       <c r="C5" t="s">
         <v>9</v>
       </c>
-      <c r="D5" t="s">
-        <v>28</v>
+      <c r="D5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1564,8 +1557,8 @@
       <c r="C6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" t="s">
-        <v>28</v>
+      <c r="D6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1578,8 +1571,8 @@
       <c r="C7" t="s">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
-        <v>28</v>
+      <c r="D7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1592,8 +1585,8 @@
       <c r="C8" t="s">
         <v>5</v>
       </c>
-      <c r="D8" t="s">
-        <v>28</v>
+      <c r="D8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1606,8 +1599,8 @@
       <c r="C9" t="s">
         <v>15</v>
       </c>
-      <c r="D9" t="s">
-        <v>29</v>
+      <c r="D9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1620,8 +1613,8 @@
       <c r="C10" t="s">
         <v>5</v>
       </c>
-      <c r="D10" t="s">
-        <v>28</v>
+      <c r="D10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1634,8 +1627,8 @@
       <c r="C11" t="s">
         <v>19</v>
       </c>
-      <c r="D11" t="s">
-        <v>28</v>
+      <c r="D11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1648,8 +1641,8 @@
       <c r="C12" t="s">
         <v>5</v>
       </c>
-      <c r="D12" t="s">
-        <v>28</v>
+      <c r="D12" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1662,8 +1655,22 @@
       <c r="C13" t="s">
         <v>23</v>
       </c>
-      <c r="D13" t="s">
-        <v>28</v>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>8</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed vip25, normalo23, add week 5 for vip26
</commit_message>
<xml_diff>
--- a/data/vip2025.xlsx
+++ b/data/vip2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805FC4C3-AFAA-9041-8519-5BC3B6164E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE00C2A-79AD-734A-920B-9AB7526FC16C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="760" windowWidth="33720" windowHeight="17820" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="560" yWindow="1940" windowWidth="18620" windowHeight="21020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="28">
   <si>
     <t>left</t>
   </si>
@@ -82,9 +82,6 @@
     <t>Nelly</t>
   </si>
   <si>
-    <t>Olli</t>
-  </si>
-  <si>
     <t>Sandra</t>
   </si>
   <si>
@@ -107,6 +104,9 @@
   </si>
   <si>
     <t>result</t>
+  </si>
+  <si>
+    <t>Oliver</t>
   </si>
 </sst>
 </file>
@@ -1031,28 +1031,28 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
         <v>20</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
         <v>22</v>
-      </c>
-      <c r="B11" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1102,13 +1102,13 @@
         <v>18</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1122,7 +1122,7 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
         <v>4</v>
@@ -1131,10 +1131,10 @@
         <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I2" t="s">
         <v>11</v>
@@ -1154,22 +1154,22 @@
         <v>17</v>
       </c>
       <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
         <v>23</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
       </c>
       <c r="E3" t="s">
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
         <v>7</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I3" t="s">
         <v>11</v>
@@ -1183,7 +1183,7 @@
     </row>
     <row r="4" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -1192,10 +1192,10 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
         <v>13</v>
@@ -1218,19 +1218,19 @@
     </row>
     <row r="5" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F5" t="s">
         <v>15</v>
@@ -1253,19 +1253,19 @@
     </row>
     <row r="6" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
-        <v>24</v>
-      </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F6" t="s">
         <v>5</v>
@@ -1297,16 +1297,16 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s">
         <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1332,19 +1332,19 @@
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
         <v>9</v>
       </c>
       <c r="F8" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I8" t="s">
         <v>15</v>
@@ -1367,19 +1367,19 @@
         <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" t="s">
         <v>9</v>
       </c>
       <c r="F9" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G9" t="s">
         <v>4</v>
       </c>
       <c r="H9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I9" t="s">
         <v>15</v>
@@ -1399,16 +1399,16 @@
         <v>13</v>
       </c>
       <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s">
         <v>23</v>
-      </c>
-      <c r="D10" t="s">
-        <v>24</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G10" t="s">
         <v>7</v>
@@ -1420,7 +1420,7 @@
         <v>15</v>
       </c>
       <c r="J10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K10">
         <v>4</v>
@@ -1431,22 +1431,22 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s">
         <v>13</v>
       </c>
       <c r="G11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H11" t="s">
         <v>4</v>
@@ -1471,7 +1471,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -1479,7 +1479,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1488,46 +1488,46 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="D3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
@@ -1538,10 +1538,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -1549,13 +1549,13 @@
     </row>
     <row r="6" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -1563,27 +1563,27 @@
     </row>
     <row r="7" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>
@@ -1591,86 +1591,58 @@
     </row>
     <row r="9" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>15</v>
-      </c>
       <c r="D9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="D10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
         <v>7</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" t="s">
-        <v>5</v>
       </c>
       <c r="D12" t="b">
         <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>8</v>
-      </c>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>8</v>
-      </c>
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" t="b">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1731,7 +1703,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -1739,7 +1711,7 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -1747,7 +1719,7 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -1763,7 +1735,7 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -1776,7 +1748,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
         <v>15</v>
@@ -1784,7 +1756,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>

</xml_diff>